<commit_message>
- create animation for piece movement - add special moves (en passant, castling, queen promotion) - improve ui experience (board indexes, border for white team)
</commit_message>
<xml_diff>
--- a/Tools/languages.xlsx
+++ b/Tools/languages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/chess/Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F69411-D919-9241-BAED-07D58ADC8E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518B613D-4ABD-0E4B-8A90-3565CEFBA5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15840" xr2:uid="{E6764379-1D78-984F-8202-F6CD8653F853}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
   <si>
     <t>Key</t>
   </si>
@@ -122,13 +122,22 @@
     <t>Lịch sử</t>
   </si>
   <si>
-    <t>page.home</t>
-  </si>
-  <si>
-    <t>page.history</t>
-  </si>
-  <si>
-    <t>page.about</t>
+    <t>page.home.title</t>
+  </si>
+  <si>
+    <t>page.history.title</t>
+  </si>
+  <si>
+    <t>page.about.title</t>
+  </si>
+  <si>
+    <t>home.turn.title</t>
+  </si>
+  <si>
+    <t>Turn</t>
+  </si>
+  <si>
+    <t>Lượt đánh</t>
   </si>
 </sst>
 </file>
@@ -695,10 +704,16 @@
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+    <row r="16" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>

</xml_diff>

<commit_message>
layout with side menu
</commit_message>
<xml_diff>
--- a/Tools/languages.xlsx
+++ b/Tools/languages.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/chess/Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518B613D-4ABD-0E4B-8A90-3565CEFBA5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3D9696-AA85-D14D-B265-6F0B144E45C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15840" xr2:uid="{E6764379-1D78-984F-8202-F6CD8653F853}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>Key</t>
   </si>
@@ -98,9 +98,6 @@
     <t>menu.home</t>
   </si>
   <si>
-    <t>menu.about</t>
-  </si>
-  <si>
     <t>Home</t>
   </si>
   <si>
@@ -113,9 +110,6 @@
     <t>Thông tin</t>
   </si>
   <si>
-    <t>menu.history</t>
-  </si>
-  <si>
     <t>History</t>
   </si>
   <si>
@@ -138,6 +132,15 @@
   </si>
   <si>
     <t>Lượt đánh</t>
+  </si>
+  <si>
+    <t>menu.logout</t>
+  </si>
+  <si>
+    <t>Logout</t>
+  </si>
+  <si>
+    <t>Đăng xuất</t>
   </si>
 </sst>
 </file>
@@ -543,7 +546,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A972E6DD-A464-F34F-8D77-960075701A8D}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:C473"/>
+  <dimension ref="A1:C472"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.5" style="2" bestFit="1" customWidth="1"/>
@@ -575,35 +578,35 @@
     </row>
     <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.2">
@@ -622,98 +625,92 @@
         <v>19</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="16" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+    <row r="14" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>33</v>
-      </c>
+    </row>
+    <row r="16" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
     </row>
     <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
@@ -1146,7 +1143,7 @@
       <c r="C102" s="3"/>
     </row>
     <row r="103" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A103" s="1"/>
+      <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
     </row>
@@ -1156,7 +1153,7 @@
       <c r="C104" s="3"/>
     </row>
     <row r="105" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A105" s="3"/>
+      <c r="A105" s="1"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
     </row>
@@ -1487,8 +1484,8 @@
     </row>
     <row r="171" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A171" s="1"/>
-      <c r="B171" s="3"/>
-      <c r="C171" s="3"/>
+      <c r="B171" s="4"/>
+      <c r="C171" s="4"/>
     </row>
     <row r="172" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A172" s="1"/>
@@ -1512,8 +1509,8 @@
     </row>
     <row r="176" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A176" s="1"/>
-      <c r="B176" s="4"/>
-      <c r="C176" s="4"/>
+      <c r="B176" s="3"/>
+      <c r="C176" s="3"/>
     </row>
     <row r="177" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A177" s="1"/>
@@ -1552,8 +1549,8 @@
     </row>
     <row r="184" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A184" s="1"/>
-      <c r="B184" s="3"/>
-      <c r="C184" s="3"/>
+      <c r="B184" s="4"/>
+      <c r="C184" s="4"/>
     </row>
     <row r="185" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A185" s="1"/>
@@ -1577,8 +1574,8 @@
     </row>
     <row r="189" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A189" s="1"/>
-      <c r="B189" s="4"/>
-      <c r="C189" s="4"/>
+      <c r="B189" s="3"/>
+      <c r="C189" s="3"/>
     </row>
     <row r="190" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A190" s="1"/>
@@ -2272,12 +2269,12 @@
     </row>
     <row r="328" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A328" s="1"/>
-      <c r="B328" s="3"/>
+      <c r="B328" s="1"/>
       <c r="C328" s="3"/>
     </row>
     <row r="329" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A329" s="1"/>
-      <c r="B329" s="1"/>
+      <c r="B329" s="3"/>
       <c r="C329" s="3"/>
     </row>
     <row r="330" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2447,7 +2444,7 @@
     </row>
     <row r="363" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A363" s="1"/>
-      <c r="B363" s="3"/>
+      <c r="B363" s="1"/>
       <c r="C363" s="3"/>
     </row>
     <row r="364" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2457,7 +2454,7 @@
     </row>
     <row r="365" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A365" s="1"/>
-      <c r="B365" s="1"/>
+      <c r="B365" s="3"/>
       <c r="C365" s="3"/>
     </row>
     <row r="366" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2822,13 +2819,13 @@
     </row>
     <row r="438" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A438" s="1"/>
-      <c r="B438" s="3"/>
-      <c r="C438" s="3"/>
+      <c r="B438" s="1"/>
+      <c r="C438" s="1"/>
     </row>
     <row r="439" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A439" s="1"/>
-      <c r="B439" s="1"/>
-      <c r="C439" s="1"/>
+      <c r="B439" s="3"/>
+      <c r="C439" s="3"/>
     </row>
     <row r="440" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A440" s="1"/>
@@ -2887,8 +2884,8 @@
     </row>
     <row r="451" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A451" s="1"/>
-      <c r="B451" s="3"/>
-      <c r="C451" s="3"/>
+      <c r="B451" s="1"/>
+      <c r="C451" s="1"/>
     </row>
     <row r="452" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A452" s="1"/>
@@ -2912,8 +2909,8 @@
     </row>
     <row r="456" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A456" s="1"/>
-      <c r="B456" s="1"/>
-      <c r="C456" s="1"/>
+      <c r="B456" s="3"/>
+      <c r="C456" s="3"/>
     </row>
     <row r="457" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A457" s="1"/>
@@ -2987,22 +2984,17 @@
     </row>
     <row r="471" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A471" s="1"/>
-      <c r="B471" s="3"/>
-      <c r="C471" s="3"/>
+      <c r="B471" s="1"/>
+      <c r="C471" s="1"/>
     </row>
     <row r="472" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A472" s="1"/>
       <c r="B472" s="1"/>
       <c r="C472" s="1"/>
     </row>
-    <row r="473" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A473" s="1"/>
-      <c r="B473" s="1"/>
-      <c r="C473" s="1"/>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A280:C284">
-    <sortCondition ref="A280:A284"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A279:C283">
+    <sortCondition ref="A279:A283"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
setup hamburger button for mobile mode
</commit_message>
<xml_diff>
--- a/Tools/languages.xlsx
+++ b/Tools/languages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/chess/Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3D9696-AA85-D14D-B265-6F0B144E45C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46057BD-896D-9347-B9EC-C00727019DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15840" xr2:uid="{E6764379-1D78-984F-8202-F6CD8653F853}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="41">
   <si>
     <t>Key</t>
   </si>
@@ -47,15 +47,6 @@
     <t>Vietnamese</t>
   </si>
   <si>
-    <t>This field is required</t>
-  </si>
-  <si>
-    <t>Trường này bắt buộc nhập</t>
-  </si>
-  <si>
-    <t>constant.field-required</t>
-  </si>
-  <si>
     <t>settings.header</t>
   </si>
   <si>
@@ -141,6 +132,33 @@
   </si>
   <si>
     <t>Đăng xuất</t>
+  </si>
+  <si>
+    <t>Chess game</t>
+  </si>
+  <si>
+    <t>Cờ vua</t>
+  </si>
+  <si>
+    <t>menu.app-name</t>
+  </si>
+  <si>
+    <t>menu.users</t>
+  </si>
+  <si>
+    <t>Users</t>
+  </si>
+  <si>
+    <t>Người dùng</t>
+  </si>
+  <si>
+    <t>Analytic</t>
+  </si>
+  <si>
+    <t>Phân tích</t>
+  </si>
+  <si>
+    <t>menu.analytics</t>
   </si>
 </sst>
 </file>
@@ -546,7 +564,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A972E6DD-A464-F34F-8D77-960075701A8D}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:C472"/>
+  <dimension ref="A1:C474"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.5" style="2" bestFit="1" customWidth="1"/>
@@ -567,21 +585,21 @@
     </row>
     <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>22</v>
@@ -589,122 +607,128 @@
     </row>
     <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -712,10 +736,16 @@
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+    <row r="17" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="18" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
@@ -1143,22 +1173,22 @@
       <c r="C102" s="3"/>
     </row>
     <row r="103" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A103" s="3"/>
+      <c r="A103" s="1"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
     </row>
     <row r="104" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A104" s="3"/>
+      <c r="A104" s="1"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
     </row>
     <row r="105" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A105" s="1"/>
+      <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
     </row>
     <row r="106" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A106" s="1"/>
+      <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
     </row>
@@ -1484,13 +1514,13 @@
     </row>
     <row r="171" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A171" s="1"/>
-      <c r="B171" s="4"/>
-      <c r="C171" s="4"/>
+      <c r="B171" s="3"/>
+      <c r="C171" s="3"/>
     </row>
     <row r="172" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A172" s="1"/>
-      <c r="B172" s="4"/>
-      <c r="C172" s="4"/>
+      <c r="B172" s="3"/>
+      <c r="C172" s="3"/>
     </row>
     <row r="173" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A173" s="1"/>
@@ -1509,13 +1539,13 @@
     </row>
     <row r="176" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A176" s="1"/>
-      <c r="B176" s="3"/>
-      <c r="C176" s="3"/>
+      <c r="B176" s="4"/>
+      <c r="C176" s="4"/>
     </row>
     <row r="177" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A177" s="1"/>
-      <c r="B177" s="3"/>
-      <c r="C177" s="3"/>
+      <c r="B177" s="4"/>
+      <c r="C177" s="4"/>
     </row>
     <row r="178" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A178" s="1"/>
@@ -1549,13 +1579,13 @@
     </row>
     <row r="184" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A184" s="1"/>
-      <c r="B184" s="4"/>
-      <c r="C184" s="4"/>
+      <c r="B184" s="3"/>
+      <c r="C184" s="3"/>
     </row>
     <row r="185" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A185" s="1"/>
-      <c r="B185" s="4"/>
-      <c r="C185" s="4"/>
+      <c r="B185" s="3"/>
+      <c r="C185" s="3"/>
     </row>
     <row r="186" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A186" s="1"/>
@@ -1574,13 +1604,13 @@
     </row>
     <row r="189" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A189" s="1"/>
-      <c r="B189" s="3"/>
-      <c r="C189" s="3"/>
+      <c r="B189" s="4"/>
+      <c r="C189" s="4"/>
     </row>
     <row r="190" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A190" s="1"/>
-      <c r="B190" s="3"/>
-      <c r="C190" s="3"/>
+      <c r="B190" s="4"/>
+      <c r="C190" s="4"/>
     </row>
     <row r="191" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A191" s="1"/>
@@ -2269,7 +2299,7 @@
     </row>
     <row r="328" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A328" s="1"/>
-      <c r="B328" s="1"/>
+      <c r="B328" s="3"/>
       <c r="C328" s="3"/>
     </row>
     <row r="329" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2279,7 +2309,7 @@
     </row>
     <row r="330" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A330" s="1"/>
-      <c r="B330" s="3"/>
+      <c r="B330" s="1"/>
       <c r="C330" s="3"/>
     </row>
     <row r="331" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2444,22 +2474,22 @@
     </row>
     <row r="363" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A363" s="1"/>
-      <c r="B363" s="1"/>
+      <c r="B363" s="3"/>
       <c r="C363" s="3"/>
     </row>
     <row r="364" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A364" s="1"/>
-      <c r="B364" s="1"/>
+      <c r="B364" s="3"/>
       <c r="C364" s="3"/>
     </row>
     <row r="365" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A365" s="1"/>
-      <c r="B365" s="3"/>
+      <c r="B365" s="1"/>
       <c r="C365" s="3"/>
     </row>
     <row r="366" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A366" s="1"/>
-      <c r="B366" s="3"/>
+      <c r="B366" s="1"/>
       <c r="C366" s="3"/>
     </row>
     <row r="367" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2819,8 +2849,8 @@
     </row>
     <row r="438" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A438" s="1"/>
-      <c r="B438" s="1"/>
-      <c r="C438" s="1"/>
+      <c r="B438" s="3"/>
+      <c r="C438" s="3"/>
     </row>
     <row r="439" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A439" s="1"/>
@@ -2829,8 +2859,8 @@
     </row>
     <row r="440" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A440" s="1"/>
-      <c r="B440" s="3"/>
-      <c r="C440" s="3"/>
+      <c r="B440" s="1"/>
+      <c r="C440" s="1"/>
     </row>
     <row r="441" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A441" s="1"/>
@@ -2884,13 +2914,13 @@
     </row>
     <row r="451" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A451" s="1"/>
-      <c r="B451" s="1"/>
-      <c r="C451" s="1"/>
+      <c r="B451" s="3"/>
+      <c r="C451" s="3"/>
     </row>
     <row r="452" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A452" s="1"/>
-      <c r="B452" s="1"/>
-      <c r="C452" s="1"/>
+      <c r="B452" s="3"/>
+      <c r="C452" s="3"/>
     </row>
     <row r="453" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A453" s="1"/>
@@ -2909,13 +2939,13 @@
     </row>
     <row r="456" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A456" s="1"/>
-      <c r="B456" s="3"/>
-      <c r="C456" s="3"/>
+      <c r="B456" s="1"/>
+      <c r="C456" s="1"/>
     </row>
     <row r="457" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A457" s="1"/>
-      <c r="B457" s="3"/>
-      <c r="C457" s="3"/>
+      <c r="B457" s="1"/>
+      <c r="C457" s="1"/>
     </row>
     <row r="458" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A458" s="1"/>
@@ -2984,17 +3014,27 @@
     </row>
     <row r="471" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A471" s="1"/>
-      <c r="B471" s="1"/>
-      <c r="C471" s="1"/>
+      <c r="B471" s="3"/>
+      <c r="C471" s="3"/>
     </row>
     <row r="472" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A472" s="1"/>
-      <c r="B472" s="1"/>
-      <c r="C472" s="1"/>
+      <c r="B472" s="3"/>
+      <c r="C472" s="3"/>
+    </row>
+    <row r="473" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A473" s="1"/>
+      <c r="B473" s="1"/>
+      <c r="C473" s="1"/>
+    </row>
+    <row r="474" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A474" s="1"/>
+      <c r="B474" s="1"/>
+      <c r="C474" s="1"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A279:C283">
-    <sortCondition ref="A279:A283"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A281:C285">
+    <sortCondition ref="A281:A285"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
- handle more behaviors - add ui experiments - layout components for pages
- handle more behaviors
- add ui experiments
- layout components for pages
</commit_message>
<xml_diff>
--- a/Tools/languages.xlsx
+++ b/Tools/languages.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/projects/hieunm/chess/Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518B613D-4ABD-0E4B-8A90-3565CEFBA5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F7D354-4B24-3243-AF79-DFB6D259C079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15840" xr2:uid="{E6764379-1D78-984F-8202-F6CD8653F853}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="49">
   <si>
     <t>Key</t>
   </si>
@@ -47,15 +47,6 @@
     <t>Vietnamese</t>
   </si>
   <si>
-    <t>This field is required</t>
-  </si>
-  <si>
-    <t>Trường này bắt buộc nhập</t>
-  </si>
-  <si>
-    <t>constant.field-required</t>
-  </si>
-  <si>
     <t>settings.header</t>
   </si>
   <si>
@@ -98,9 +89,6 @@
     <t>menu.home</t>
   </si>
   <si>
-    <t>menu.about</t>
-  </si>
-  <si>
     <t>Home</t>
   </si>
   <si>
@@ -113,9 +101,6 @@
     <t>Thông tin</t>
   </si>
   <si>
-    <t>menu.history</t>
-  </si>
-  <si>
     <t>History</t>
   </si>
   <si>
@@ -138,6 +123,66 @@
   </si>
   <si>
     <t>Lượt đánh</t>
+  </si>
+  <si>
+    <t>menu.logout</t>
+  </si>
+  <si>
+    <t>Logout</t>
+  </si>
+  <si>
+    <t>Đăng xuất</t>
+  </si>
+  <si>
+    <t>Chess game</t>
+  </si>
+  <si>
+    <t>Cờ vua</t>
+  </si>
+  <si>
+    <t>menu.app-name</t>
+  </si>
+  <si>
+    <t>menu.users</t>
+  </si>
+  <si>
+    <t>Users</t>
+  </si>
+  <si>
+    <t>Người dùng</t>
+  </si>
+  <si>
+    <t>Analytic</t>
+  </si>
+  <si>
+    <t>Phân tích</t>
+  </si>
+  <si>
+    <t>menu.analytics</t>
+  </si>
+  <si>
+    <t>popup.confirm.ok</t>
+  </si>
+  <si>
+    <t>popup.confirm.cancel</t>
+  </si>
+  <si>
+    <t>Ok</t>
+  </si>
+  <si>
+    <t>Cancel</t>
+  </si>
+  <si>
+    <t>Huỷ</t>
+  </si>
+  <si>
+    <t>game.king.captured</t>
+  </si>
+  <si>
+    <t>King has been captured. Game over</t>
+  </si>
+  <si>
+    <t>Vua đã bị bắt. Game kết thúc</t>
   </si>
 </sst>
 </file>
@@ -543,7 +588,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A972E6DD-A464-F34F-8D77-960075701A8D}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:C473"/>
+  <dimension ref="A1:C475"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.5" style="2" bestFit="1" customWidth="1"/>
@@ -564,171 +609,195 @@
     </row>
     <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>10</v>
-      </c>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="16" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-    </row>
-    <row r="18" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-    </row>
-    <row r="19" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="20" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
@@ -1151,22 +1220,22 @@
       <c r="C103" s="3"/>
     </row>
     <row r="104" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A104" s="3"/>
+      <c r="A104" s="1"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
     </row>
     <row r="105" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A105" s="3"/>
+      <c r="A105" s="1"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
     </row>
     <row r="106" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A106" s="1"/>
+      <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
     </row>
     <row r="107" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A107" s="1"/>
+      <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
     </row>
@@ -1492,13 +1561,13 @@
     </row>
     <row r="172" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A172" s="1"/>
-      <c r="B172" s="4"/>
-      <c r="C172" s="4"/>
+      <c r="B172" s="3"/>
+      <c r="C172" s="3"/>
     </row>
     <row r="173" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A173" s="1"/>
-      <c r="B173" s="4"/>
-      <c r="C173" s="4"/>
+      <c r="B173" s="3"/>
+      <c r="C173" s="3"/>
     </row>
     <row r="174" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A174" s="1"/>
@@ -1517,13 +1586,13 @@
     </row>
     <row r="177" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A177" s="1"/>
-      <c r="B177" s="3"/>
-      <c r="C177" s="3"/>
+      <c r="B177" s="4"/>
+      <c r="C177" s="4"/>
     </row>
     <row r="178" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A178" s="1"/>
-      <c r="B178" s="3"/>
-      <c r="C178" s="3"/>
+      <c r="B178" s="4"/>
+      <c r="C178" s="4"/>
     </row>
     <row r="179" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A179" s="1"/>
@@ -1557,13 +1626,13 @@
     </row>
     <row r="185" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A185" s="1"/>
-      <c r="B185" s="4"/>
-      <c r="C185" s="4"/>
+      <c r="B185" s="3"/>
+      <c r="C185" s="3"/>
     </row>
     <row r="186" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A186" s="1"/>
-      <c r="B186" s="4"/>
-      <c r="C186" s="4"/>
+      <c r="B186" s="3"/>
+      <c r="C186" s="3"/>
     </row>
     <row r="187" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A187" s="1"/>
@@ -1582,13 +1651,13 @@
     </row>
     <row r="190" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A190" s="1"/>
-      <c r="B190" s="3"/>
-      <c r="C190" s="3"/>
+      <c r="B190" s="4"/>
+      <c r="C190" s="4"/>
     </row>
     <row r="191" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A191" s="1"/>
-      <c r="B191" s="3"/>
-      <c r="C191" s="3"/>
+      <c r="B191" s="4"/>
+      <c r="C191" s="4"/>
     </row>
     <row r="192" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A192" s="1"/>
@@ -2277,7 +2346,7 @@
     </row>
     <row r="329" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A329" s="1"/>
-      <c r="B329" s="1"/>
+      <c r="B329" s="3"/>
       <c r="C329" s="3"/>
     </row>
     <row r="330" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2287,7 +2356,7 @@
     </row>
     <row r="331" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A331" s="1"/>
-      <c r="B331" s="3"/>
+      <c r="B331" s="1"/>
       <c r="C331" s="3"/>
     </row>
     <row r="332" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2452,22 +2521,22 @@
     </row>
     <row r="364" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A364" s="1"/>
-      <c r="B364" s="1"/>
+      <c r="B364" s="3"/>
       <c r="C364" s="3"/>
     </row>
     <row r="365" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A365" s="1"/>
-      <c r="B365" s="1"/>
+      <c r="B365" s="3"/>
       <c r="C365" s="3"/>
     </row>
     <row r="366" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A366" s="1"/>
-      <c r="B366" s="3"/>
+      <c r="B366" s="1"/>
       <c r="C366" s="3"/>
     </row>
     <row r="367" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A367" s="1"/>
-      <c r="B367" s="3"/>
+      <c r="B367" s="1"/>
       <c r="C367" s="3"/>
     </row>
     <row r="368" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -2827,8 +2896,8 @@
     </row>
     <row r="439" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A439" s="1"/>
-      <c r="B439" s="1"/>
-      <c r="C439" s="1"/>
+      <c r="B439" s="3"/>
+      <c r="C439" s="3"/>
     </row>
     <row r="440" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A440" s="1"/>
@@ -2837,8 +2906,8 @@
     </row>
     <row r="441" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A441" s="1"/>
-      <c r="B441" s="3"/>
-      <c r="C441" s="3"/>
+      <c r="B441" s="1"/>
+      <c r="C441" s="1"/>
     </row>
     <row r="442" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A442" s="1"/>
@@ -2892,13 +2961,13 @@
     </row>
     <row r="452" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A452" s="1"/>
-      <c r="B452" s="1"/>
-      <c r="C452" s="1"/>
+      <c r="B452" s="3"/>
+      <c r="C452" s="3"/>
     </row>
     <row r="453" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A453" s="1"/>
-      <c r="B453" s="1"/>
-      <c r="C453" s="1"/>
+      <c r="B453" s="3"/>
+      <c r="C453" s="3"/>
     </row>
     <row r="454" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A454" s="1"/>
@@ -2917,13 +2986,13 @@
     </row>
     <row r="457" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A457" s="1"/>
-      <c r="B457" s="3"/>
-      <c r="C457" s="3"/>
+      <c r="B457" s="1"/>
+      <c r="C457" s="1"/>
     </row>
     <row r="458" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A458" s="1"/>
-      <c r="B458" s="3"/>
-      <c r="C458" s="3"/>
+      <c r="B458" s="1"/>
+      <c r="C458" s="1"/>
     </row>
     <row r="459" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A459" s="1"/>
@@ -2992,17 +3061,27 @@
     </row>
     <row r="472" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A472" s="1"/>
-      <c r="B472" s="1"/>
-      <c r="C472" s="1"/>
+      <c r="B472" s="3"/>
+      <c r="C472" s="3"/>
     </row>
     <row r="473" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A473" s="1"/>
-      <c r="B473" s="1"/>
-      <c r="C473" s="1"/>
+      <c r="B473" s="3"/>
+      <c r="C473" s="3"/>
+    </row>
+    <row r="474" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A474" s="1"/>
+      <c r="B474" s="1"/>
+      <c r="C474" s="1"/>
+    </row>
+    <row r="475" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A475" s="1"/>
+      <c r="B475" s="1"/>
+      <c r="C475" s="1"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A280:C284">
-    <sortCondition ref="A280:A284"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A282:C286">
+    <sortCondition ref="A282:A286"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>